<commit_message>
SOV 38ALT Main Gate Perimiter VA INTRUSION => SOV 38ALT Main Gate Perimeter VA INTRUSION
</commit_message>
<xml_diff>
--- a/apigw/docs/VA_ForWebHookCreation.xlsx
+++ b/apigw/docs/VA_ForWebHookCreation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\cde\apigw\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB8F975-8749-4CE2-9D96-0409ABB35233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2E97F7-5D17-4411-B122-880AC2A951D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="98">
   <si>
     <t>#</t>
   </si>
@@ -266,9 +266,6 @@
     <t>curl -i -X GET http://10.65.51.252:8088/va/sov-38alt-l5-o-s-cyber-room-loitering -u "vizzio@imops.local:xAJHkkm7m3V5MhtF0xGM"</t>
   </si>
   <si>
-    <t>SOV 38ALT Main Gate Perimiter</t>
-  </si>
-  <si>
     <t>SOV_38ALT_Main_Gate_Perimeter</t>
   </si>
   <si>
@@ -329,10 +326,7 @@
     <t>SOV 38ALT Side Fencing VA SMOKING</t>
   </si>
   <si>
-    <t>if one by one okay</t>
-  </si>
-  <si>
-    <t>combine 15 + 16 playback would failed</t>
+    <t>SOV 38ALT Main Gate Perimeter</t>
   </si>
 </sst>
 </file>
@@ -439,7 +433,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -466,10 +460,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -809,22 +800,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N22"/>
-  <sheetFormatPr defaultRowHeight="21.65" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21.6" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.54296875" customWidth="1"/>
-    <col min="2" max="2" width="20.54296875" customWidth="1"/>
-    <col min="3" max="3" width="35.453125" customWidth="1"/>
-    <col min="4" max="4" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="80.453125" customWidth="1"/>
-    <col min="6" max="6" width="14.81640625" customWidth="1"/>
-    <col min="9" max="9" width="12.7265625" customWidth="1"/>
-    <col min="10" max="10" width="34.1796875" customWidth="1"/>
-    <col min="11" max="11" width="32.1796875" customWidth="1"/>
-    <col min="12" max="12" width="121.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
+    <col min="4" max="4" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="80.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="34.140625" customWidth="1"/>
+    <col min="11" max="11" width="32.140625" customWidth="1"/>
+    <col min="12" max="12" width="121.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="24" style="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -862,10 +853,10 @@
         <v>11</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -903,7 +894,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -942,7 +933,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -981,7 +972,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -1020,7 +1011,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -1034,7 +1025,7 @@
         <v>32</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
@@ -1062,7 +1053,7 @@
       </c>
       <c r="N6" s="6"/>
     </row>
-    <row r="7" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>6</v>
       </c>
@@ -1089,7 +1080,7 @@
         <v>2</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>12</v>
@@ -1101,7 +1092,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>7</v>
       </c>
@@ -1128,7 +1119,7 @@
         <v>2</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>12</v>
@@ -1140,7 +1131,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>8</v>
       </c>
@@ -1167,7 +1158,7 @@
         <v>2</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>12</v>
@@ -1179,7 +1170,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>9</v>
       </c>
@@ -1206,7 +1197,7 @@
         <v>2</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>12</v>
@@ -1218,7 +1209,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>10</v>
       </c>
@@ -1245,7 +1236,7 @@
         <v>1</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>47</v>
@@ -1257,7 +1248,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>11</v>
       </c>
@@ -1284,7 +1275,7 @@
         <v>1</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>22</v>
@@ -1296,7 +1287,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>12</v>
       </c>
@@ -1323,7 +1314,7 @@
         <v>1</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>27</v>
@@ -1335,7 +1326,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>13</v>
       </c>
@@ -1362,7 +1353,7 @@
         <v>4</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>12</v>
@@ -1374,7 +1365,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>14</v>
       </c>
@@ -1401,7 +1392,7 @@
         <v>2</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>12</v>
@@ -1412,12 +1403,10 @@
       <c r="M15" s="12">
         <v>111</v>
       </c>
-      <c r="N15" s="15" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="16">
+      <c r="N15" s="14"/>
+    </row>
+    <row r="16" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1443,7 +1432,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>12</v>
@@ -1452,14 +1441,12 @@
         <v>61</v>
       </c>
       <c r="M16" s="12">
-        <v>110</v>
-      </c>
-      <c r="N16" s="15" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="16">
+        <v>111</v>
+      </c>
+      <c r="N16" s="14"/>
+    </row>
+    <row r="17" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7">
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -1485,7 +1472,7 @@
         <v>2</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K17" s="3" t="s">
         <v>12</v>
@@ -1494,10 +1481,10 @@
         <v>64</v>
       </c>
       <c r="M17" s="12">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
         <v>17</v>
       </c>
@@ -1524,7 +1511,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>12</v>
@@ -1532,10 +1519,12 @@
       <c r="L18" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="M18" s="12"/>
-    </row>
-    <row r="19" spans="1:13" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="14">
+      <c r="M18" s="12">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15">
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -1561,7 +1550,7 @@
         <v>1</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>12</v>
@@ -1569,10 +1558,12 @@
       <c r="L19" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="M19" s="12"/>
-    </row>
-    <row r="20" spans="1:13" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="14">
+      <c r="M19" s="12">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7">
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -1598,7 +1589,7 @@
         <v>2</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>12</v>
@@ -1606,10 +1597,12 @@
       <c r="L20" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="M20" s="12"/>
-    </row>
-    <row r="21" spans="1:13" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="14">
+      <c r="M20" s="12">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -1635,7 +1628,7 @@
         <v>2</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>12</v>
@@ -1643,20 +1636,22 @@
       <c r="L21" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="M21" s="12"/>
-    </row>
-    <row r="22" spans="1:13" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="14">
+      <c r="M21" s="12">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7">
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="3">
@@ -1672,15 +1667,17 @@
         <v>1</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>47</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="M22" s="12"/>
+        <v>79</v>
+      </c>
+      <c r="M22" s="12">
+        <v>111</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
complete proscalar option c
</commit_message>
<xml_diff>
--- a/apigw/docs/VA_ForWebHookCreation.xlsx
+++ b/apigw/docs/VA_ForWebHookCreation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\cde\apigw\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2E97F7-5D17-4411-B122-880AC2A951D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469F0A64-911B-4045-9A32-5B2AF2B2CB60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -374,7 +374,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -384,12 +384,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -433,7 +427,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -461,9 +455,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1524,7 +1515,7 @@
       </c>
     </row>
     <row r="19" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="7">
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -1559,7 +1550,7 @@
         <v>70</v>
       </c>
       <c r="M19" s="12">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>